<commit_message>
إنشاء شيت جديد 'CLX1' مع 5 أعمدة by admin at 2026-03-06 14:39:29
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="BOP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="CLX1" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -472,4 +473,45 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>رقم الماكينه</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>الحدث</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>التصحيح</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>تم بواسطه</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
إنشاء شيت جديد 'CLX2' مع 5 أعمدة by admin at 2026-03-06 14:39:35
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="BOP" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="CLX1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CLX2" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -514,4 +515,45 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>رقم الماكينه</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>الحدث</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>التصحيح</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>تم بواسطه</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
إنشاء شيت جديد 'MIX1' مع 5 أعمدة by admin at 2026-03-06 14:39:45
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -11,6 +11,7 @@
     <sheet name="BOP" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="CLX1" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="CLX2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="MIX1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -556,4 +557,45 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>رقم الماكينه</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>الحدث</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>التصحيح</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>تم بواسطه</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
إنشاء شيت جديد 'MIX2' مع 5 أعمدة by admin at 2026-03-06 14:39:52
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -12,6 +12,7 @@
     <sheet name="CLX1" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="CLX2" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="MIX1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="MIX2" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -598,4 +599,45 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>رقم الماكينه</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>الحدث</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>التصحيح</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>تم بواسطه</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
إنشاء شيت جديد 'CLU1' مع 5 أعمدة by admin at 2026-03-06 14:40:02
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -13,6 +13,7 @@
     <sheet name="CLX2" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="MIX1" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="MIX2" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CLU1" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -640,4 +641,45 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>رقم الماكينه</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>الحدث</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>التصحيح</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>تم بواسطه</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
إنشاء شيت جديد 'CLU2' مع 5 أعمدة by admin at 2026-03-06 14:40:07
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -14,6 +14,7 @@
     <sheet name="MIX1" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="MIX2" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="CLU1" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="CLU2" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -682,4 +683,45 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>رقم الماكينه</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>الحدث</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>التصحيح</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>تم بواسطه</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
إنشاء شيت جديد 'TS_T51' مع 5 أعمدة by admin at 2026-03-06 14:40:21
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -15,6 +15,7 @@
     <sheet name="MIX2" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="CLU1" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="CLU2" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="TS_T51" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -724,4 +725,45 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>رقم الماكينه</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>الحدث</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>التصحيح</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>تم بواسطه</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
إنشاء شيت جديد 'TS_T52' مع 5 أعمدة by admin at 2026-03-06 14:40:30
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -16,6 +16,7 @@
     <sheet name="CLU1" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="CLU2" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="TS_T51" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="TS_T52" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -440,7 +441,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -481,7 +482,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -522,7 +523,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -563,7 +564,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -604,7 +605,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -645,7 +646,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -686,7 +687,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -727,7 +728,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -766,4 +767,45 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>رقم الماكينه</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>الحدث</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>التصحيح</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>تم بواسطه</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
إنشاء شيت جديد 'SP_MF' مع 5 أعمدة by admin at 2026-03-06 14:40:44
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -17,6 +17,7 @@
     <sheet name="CLU2" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="TS_T51" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="TS_T52" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="SP_MF" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -482,6 +483,47 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>رقم الماكينه</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>الحدث</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>التصحيح</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>تم بواسطه</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
إضافة حدث جديد في CLX1 by admin at 2026-03-06 15:35:33
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -640,6 +640,74 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>رقم الماكينه</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>الحدث</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>التصحيح</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>تم بواسطه</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>تم التركيب</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>تم التشغيل</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1\2\2024</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>م.صيام</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -675,7 +743,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -716,7 +784,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -757,7 +825,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -798,7 +866,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -839,7 +907,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -878,45 +946,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>رقم الماكينه</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>الحدث</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>التصحيح</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>التاريخ</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>تم بواسطه</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
إضافة حدث جديد في CLX1 by admin at 2026-03-06 15:35:35
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -697,6 +697,33 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>تم التركيب</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>تم التشغيل</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1\2\2024</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>م.صيام</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
إضافة حدث جديد في BOP by admin at 2026-03-07 12:28:15
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -629,6 +629,33 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>قطع سير رولات تسويه (3150)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>تم تغير سير رولات 3150</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>28/11/2024</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>م.محمد عبدالله ،حسام</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
إضافة حدث جديد في CLX1 by admin at 2026-03-07 12:29:45
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -751,6 +751,33 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>تغيير سوفت</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>تم تغيير السوفت</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1/9/2024</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>م/احمدعلي</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
إضافة حدث جديد في BOP by admin at 2026-03-07 12:30:31
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -572,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -656,6 +656,33 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>هلك عجله بلندوم ارضيه</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>تم تغير عجله بلندوم</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>13/12/2025</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>م.محمد عبدالله ،حسام،م.شحته،عمر</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
إضافة حدث جديد في MIX1 by admin at 2026-03-07 12:32:36
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -857,7 +857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -887,6 +887,33 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>صيانه شهريه</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تم تشحيم الكتاينه والتشييك علي الچونات </t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>24/7/2024</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>تيم الكرد</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
إضافة حدث جديد في MIX1 by admin at 2026-03-07 12:33:07
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -857,7 +857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -909,6 +909,33 @@
         </is>
       </c>
       <c r="E2" t="inlineStr">
+        <is>
+          <t>تيم الكرد</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>صيانه شهريه</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تم تشحيم الكتاينه والتشييك علي الچونات </t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>26/8/2024</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>تيم الكرد</t>
         </is>

</xml_diff>

<commit_message>
إضافة حدث جديد في CLU1 by admin at 2026-03-07 12:33:52
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -993,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1020,6 +1020,33 @@
       <c r="E1" s="1" t="inlineStr">
         <is>
           <t>تم بواسطه</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>تم التركيب</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>تم التشغيل</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>1/2/2024</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>م.صيام</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
إضافة حدث جديد في MIX1 by admin at 2026-03-07 12:34:32
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -857,7 +857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -936,6 +936,33 @@
         </is>
       </c>
       <c r="E3" t="inlineStr">
+        <is>
+          <t>تيم الكرد</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> حدوث حريقه</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>حدوث حريقه في غرفه رقم 10</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>4/9/2024</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>تيم الكرد</t>
         </is>

</xml_diff>

<commit_message>
إضافة حدث جديد في MIX1 by admin at 2026-03-07 12:35:48
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -857,7 +857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -963,6 +963,33 @@
         </is>
       </c>
       <c r="E4" t="inlineStr">
+        <is>
+          <t>تيم الكرد</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ثقب في خرطوم الهواء </t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تم تغيير خرطوم الهواء </t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>17/9/2024</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>تيم الكرد</t>
         </is>

</xml_diff>

<commit_message>
إضافة حدث جديد في CLU1 by admin at 2026-03-07 12:36:32
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -1047,7 +1047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1101,6 +1101,33 @@
       <c r="E2" t="inlineStr">
         <is>
           <t>م.صيام</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> حدوث حريق ف جوان مضرب تفتيح</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>تم تغير تغير چوان</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>6/11/2024</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">م.محمد عبدالله </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
إضافة حدث جديد في MIX1 by admin at 2026-03-07 12:36:35
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -857,7 +857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -990,6 +990,33 @@
         </is>
       </c>
       <c r="E5" t="inlineStr">
+        <is>
+          <t>تيم الكرد</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>صيانه شهريه</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تم تشحيم الكتاينه والتشييك علي الچونات </t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>24/10/2024</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>تيم الكرد</t>
         </is>

</xml_diff>

<commit_message>
إضافة حدث جديد في MIX1 by admin at 2026-03-07 12:36:50
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -857,7 +857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1017,6 +1017,33 @@
         </is>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>تيم الكرد</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>صيانه شهريه</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تم تشحيم الكتاينه والتشييك علي الچونات </t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>28/10/2024</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>تيم الكرد</t>
         </is>

</xml_diff>

<commit_message>
إضافة حدث جديد في CLX1 by admin at 2026-03-07 12:37:57
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -802,6 +802,33 @@
       <c r="E4" t="inlineStr">
         <is>
           <t>م/احمدعلي</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تم التركيب </t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>تم التشغيل</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>1/2/2024</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">م صيام </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
إضافة حدث جديد في MIX1 by admin at 2026-03-07 12:38:24
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1071,6 +1071,35 @@
         </is>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>تيم الكرد</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>صيانه شهريه</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تم تشحيم الكتاينه والتشييك علي الچونات 
+و تم تغيير 2 سير 1750 
+وتغيير چوان مضرب التفتيح ال 4 اتجاه الشاشه </t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>25/12/2024</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>تيم الكرد</t>
         </is>

</xml_diff>

<commit_message>
إضافة حدث جديد في MIX1 by admin at 2026-03-07 12:39:58
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -884,7 +884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1100,6 +1100,34 @@
         </is>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>تيم الكرد</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>صيانه شهريه</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>تم تشحيم الكتاينه والتشييك علي الچونات 
+وتم شد السيور</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>5/3/2026</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>تيم الكرد</t>
         </is>

</xml_diff>

<commit_message>
إضافة حدث جديد في CLU1 by admin at 2026-03-07 12:46:04
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -1185,7 +1185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1266,6 +1266,33 @@
       <c r="E3" t="inlineStr">
         <is>
           <t xml:space="preserve">م.محمد عبدالله </t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">صيانه شهريه </t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>تم تشحيم الكتينه و التشبيك علي الچونات</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>24/7/2024</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تيم الكرد </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
إضافة حدث جديد في CLU1 by admin at 2026-03-07 12:46:23
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -1185,7 +1185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1291,6 +1291,33 @@
         </is>
       </c>
       <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تيم الكرد </t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">صيانه شهريه </t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>تم تشحيم الكتينه و التشبيك علي الچونات</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>26/8/2024</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t xml:space="preserve">تيم الكرد </t>
         </is>

</xml_diff>

<commit_message>
إضافة حدث جديد في CLU1 by admin at 2026-03-07 12:46:38
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -1185,7 +1185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1318,6 +1318,33 @@
         </is>
       </c>
       <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تيم الكرد </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">صيانه شهريه </t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>تم تشحيم الكتينه و التشبيك علي الچونات</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>24/10/2024</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t xml:space="preserve">تيم الكرد </t>
         </is>

</xml_diff>

<commit_message>
إضافة حدث جديد في CLU1 by admin at 2026-03-07 12:46:51
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -1185,7 +1185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1345,6 +1345,33 @@
         </is>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تيم الكرد </t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">صيانه شهريه </t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>تم تشحيم الكتينه و التشبيك علي الچونات</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>28/11/2024</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t xml:space="preserve">تيم الكرد </t>
         </is>

</xml_diff>

<commit_message>
إضافة حدث جديد في CLU1 by admin at 2026-03-07 12:47:47
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -1185,7 +1185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1372,6 +1372,33 @@
         </is>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تيم الكرد </t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>تغيير سوفت</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>تم تغيير السوفت الي ag</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>19/4/2025</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t xml:space="preserve">تيم الكرد </t>
         </is>

</xml_diff>

<commit_message>
إضافة حدث جديد في CLU1 by admin at 2026-03-07 12:48:32
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -1185,7 +1185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1399,6 +1399,33 @@
         </is>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تيم الكرد </t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>تغيير سوفت</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>تم تغيير السوفت من ag الي ae</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>24/4/2025</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t xml:space="preserve">تيم الكرد </t>
         </is>

</xml_diff>

<commit_message>
إضافة حدث جديد في CLX1 by admin at 2026-03-14 15:49:15
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -829,6 +829,33 @@
       <c r="E5" t="inlineStr">
         <is>
           <t xml:space="preserve">م صيام </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>هلك چوان مضرب عوادم جه بلندوم مما تسبب في ارتفاع حراره وحدوث ترب</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>تم تغير چوان باستخدام فرخ لباد محلي</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>14/3/2026</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>م.عبدالله،مصطفي،حسام،رضا،اسلام</t>
         </is>
       </c>
     </row>

</xml_diff>